<commit_message>
feat: add sourced organisation presence layers
</commit_message>
<xml_diff>
--- a/web/public/downloads/templates/africa-energy-software-map-bulk-import.xlsx
+++ b/web/public/downloads/templates/africa-energy-software-map-bulk-import.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="Rb82b10258d1e480e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bulk Records" sheetId="2" r:id="R0cecd4fea2ff49c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Examples" sheetId="3" r:id="Re67ea7fe798d4fc1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Guide" sheetId="4" r:id="Rb0b380c08aa74107"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="5" r:id="R2dc76949675a4765"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R3adebde37633467b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bulk Records" sheetId="2" r:id="Rd814c16ada9548f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Examples" sheetId="3" r:id="Rdf6f692f14964f86"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Guide" sheetId="4" r:id="R279359154a43488b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="5" r:id="R0c11d94f3d204e0a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -564,8 +564,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BulkRecordsTable" displayName="BulkRecordsTable" ref="A3:AS103" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="45">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BulkRecordsTable" displayName="BulkRecordsTable" ref="A3:AV103" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="48">
     <x:tableColumn id="1" name="row_key"/>
     <x:tableColumn id="2" name="record_type"/>
     <x:tableColumn id="3" name="organisation_name"/>
@@ -611,14 +611,17 @@
     <x:tableColumn id="43" name="source_locator"/>
     <x:tableColumn id="44" name="notes"/>
     <x:tableColumn id="45" name="confirms_no_sensitive_data"/>
+    <x:tableColumn id="46" name="organisation_presence_country_iso2"/>
+    <x:tableColumn id="47" name="organisation_presence_type"/>
+    <x:tableColumn id="48" name="organisation_presence_lifecycle_status"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ExamplesTable" displayName="ExamplesTable" ref="A3:AS9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="45">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ExamplesTable" displayName="ExamplesTable" ref="A3:AV10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="48">
     <x:tableColumn id="1" name="row_key"/>
     <x:tableColumn id="2" name="record_type"/>
     <x:tableColumn id="3" name="organisation_name"/>
@@ -664,13 +667,16 @@
     <x:tableColumn id="43" name="source_locator"/>
     <x:tableColumn id="44" name="notes"/>
     <x:tableColumn id="45" name="confirms_no_sensitive_data"/>
+    <x:tableColumn id="46" name="organisation_presence_country_iso2"/>
+    <x:tableColumn id="47" name="organisation_presence_type"/>
+    <x:tableColumn id="48" name="organisation_presence_lifecycle_status"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="FieldGuideTable" displayName="FieldGuideTable" ref="A3:C48" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="FieldGuideTable" displayName="FieldGuideTable" ref="A3:C51" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="3">
     <x:tableColumn id="1" name="Field"/>
     <x:tableColumn id="2" name="Required"/>
@@ -919,7 +925,7 @@
     </x:row>
     <x:row r="4" ht="48" customHeight="1">
       <x:c r="A4" s="27" t="str">
-        <x:v>Stage organisations, software, deployments and corporate relationships. Every row remains private until its evidence and source rights are reviewed.</x:v>
+        <x:v>Stage organisations, software, deployments, corporate relationships and country presence. Every row remains private until its evidence and source rights are reviewed.</x:v>
       </x:c>
       <x:c r="B4" s="27"/>
       <x:c r="C4" s="27"/>
@@ -1088,7 +1094,7 @@
         <x:v>Examples</x:v>
       </x:c>
       <x:c r="B17" s="35" t="str">
-        <x:v>Illustrative records for all six record types; never imported.</x:v>
+        <x:v>Illustrative records for all seven record types; never imported.</x:v>
       </x:c>
       <x:c r="C17" s="26"/>
       <x:c r="D17" s="26"/>
@@ -1184,6 +1190,9 @@
     <x:col min="43" max="43" width="32" hidden="0" customWidth="1"/>
     <x:col min="44" max="44" width="32" hidden="0" customWidth="1"/>
     <x:col min="45" max="45" width="18" hidden="0" customWidth="1"/>
+    <x:col min="46" max="46" width="18" hidden="0" customWidth="1"/>
+    <x:col min="47" max="47" width="18" hidden="0" customWidth="1"/>
+    <x:col min="48" max="48" width="18" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="35" customHeight="1">
@@ -1234,6 +1243,9 @@
       <x:c r="AQ1" s="3"/>
       <x:c r="AR1" s="3"/>
       <x:c r="AS1" s="3"/>
+      <x:c r="AT1" s="3"/>
+      <x:c r="AU1" s="3"/>
+      <x:c r="AV1" s="3"/>
     </x:row>
     <x:row r="2" ht="32" customHeight="1">
       <x:c r="A2" s="17" t="str">
@@ -1283,6 +1295,9 @@
       <x:c r="AQ2" s="17"/>
       <x:c r="AR2" s="17"/>
       <x:c r="AS2" s="17"/>
+      <x:c r="AT2" s="17"/>
+      <x:c r="AU2" s="17"/>
+      <x:c r="AV2" s="17"/>
     </x:row>
     <x:row r="3" ht="48" customHeight="1">
       <x:c r="A3" s="54" t="str">
@@ -1417,8 +1432,17 @@
       <x:c r="AR3" s="58" t="str">
         <x:v>notes</x:v>
       </x:c>
-      <x:c r="AS3" s="47" t="str">
+      <x:c r="AS3" s="46" t="str">
         <x:v>confirms_no_sensitive_data</x:v>
+      </x:c>
+      <x:c r="AT3" s="46" t="str">
+        <x:v>organisation_presence_country_iso2</x:v>
+      </x:c>
+      <x:c r="AU3" s="46" t="str">
+        <x:v>organisation_presence_type</x:v>
+      </x:c>
+      <x:c r="AV3" s="47" t="str">
+        <x:v>organisation_presence_lifecycle_status</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -1466,7 +1490,10 @@
       <x:c r="AP4" s="49" t="str"/>
       <x:c r="AQ4" s="49" t="str"/>
       <x:c r="AR4" s="49" t="str"/>
-      <x:c r="AS4" s="50" t="str"/>
+      <x:c r="AS4" s="49" t="str"/>
+      <x:c r="AT4" s="49" t="str"/>
+      <x:c r="AU4" s="49" t="str"/>
+      <x:c r="AV4" s="50" t="str"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="48" t="str"/>
@@ -1513,7 +1540,10 @@
       <x:c r="AP5" s="49" t="str"/>
       <x:c r="AQ5" s="49" t="str"/>
       <x:c r="AR5" s="49" t="str"/>
-      <x:c r="AS5" s="50" t="str"/>
+      <x:c r="AS5" s="49" t="str"/>
+      <x:c r="AT5" s="49" t="str"/>
+      <x:c r="AU5" s="49" t="str"/>
+      <x:c r="AV5" s="50" t="str"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="48" t="str"/>
@@ -1560,7 +1590,10 @@
       <x:c r="AP6" s="49" t="str"/>
       <x:c r="AQ6" s="49" t="str"/>
       <x:c r="AR6" s="49" t="str"/>
-      <x:c r="AS6" s="50" t="str"/>
+      <x:c r="AS6" s="49" t="str"/>
+      <x:c r="AT6" s="49" t="str"/>
+      <x:c r="AU6" s="49" t="str"/>
+      <x:c r="AV6" s="50" t="str"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="48" t="str"/>
@@ -1607,7 +1640,10 @@
       <x:c r="AP7" s="49" t="str"/>
       <x:c r="AQ7" s="49" t="str"/>
       <x:c r="AR7" s="49" t="str"/>
-      <x:c r="AS7" s="50" t="str"/>
+      <x:c r="AS7" s="49" t="str"/>
+      <x:c r="AT7" s="49" t="str"/>
+      <x:c r="AU7" s="49" t="str"/>
+      <x:c r="AV7" s="50" t="str"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="48" t="str"/>
@@ -1654,7 +1690,10 @@
       <x:c r="AP8" s="49" t="str"/>
       <x:c r="AQ8" s="49" t="str"/>
       <x:c r="AR8" s="49" t="str"/>
-      <x:c r="AS8" s="50" t="str"/>
+      <x:c r="AS8" s="49" t="str"/>
+      <x:c r="AT8" s="49" t="str"/>
+      <x:c r="AU8" s="49" t="str"/>
+      <x:c r="AV8" s="50" t="str"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="48" t="str"/>
@@ -1701,7 +1740,10 @@
       <x:c r="AP9" s="49" t="str"/>
       <x:c r="AQ9" s="49" t="str"/>
       <x:c r="AR9" s="49" t="str"/>
-      <x:c r="AS9" s="50" t="str"/>
+      <x:c r="AS9" s="49" t="str"/>
+      <x:c r="AT9" s="49" t="str"/>
+      <x:c r="AU9" s="49" t="str"/>
+      <x:c r="AV9" s="50" t="str"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="48" t="str"/>
@@ -1748,7 +1790,10 @@
       <x:c r="AP10" s="49" t="str"/>
       <x:c r="AQ10" s="49" t="str"/>
       <x:c r="AR10" s="49" t="str"/>
-      <x:c r="AS10" s="50" t="str"/>
+      <x:c r="AS10" s="49" t="str"/>
+      <x:c r="AT10" s="49" t="str"/>
+      <x:c r="AU10" s="49" t="str"/>
+      <x:c r="AV10" s="50" t="str"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="48" t="str"/>
@@ -1795,7 +1840,10 @@
       <x:c r="AP11" s="49" t="str"/>
       <x:c r="AQ11" s="49" t="str"/>
       <x:c r="AR11" s="49" t="str"/>
-      <x:c r="AS11" s="50" t="str"/>
+      <x:c r="AS11" s="49" t="str"/>
+      <x:c r="AT11" s="49" t="str"/>
+      <x:c r="AU11" s="49" t="str"/>
+      <x:c r="AV11" s="50" t="str"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="48" t="str"/>
@@ -1842,7 +1890,10 @@
       <x:c r="AP12" s="49" t="str"/>
       <x:c r="AQ12" s="49" t="str"/>
       <x:c r="AR12" s="49" t="str"/>
-      <x:c r="AS12" s="50" t="str"/>
+      <x:c r="AS12" s="49" t="str"/>
+      <x:c r="AT12" s="49" t="str"/>
+      <x:c r="AU12" s="49" t="str"/>
+      <x:c r="AV12" s="50" t="str"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="48" t="str"/>
@@ -1889,7 +1940,10 @@
       <x:c r="AP13" s="49" t="str"/>
       <x:c r="AQ13" s="49" t="str"/>
       <x:c r="AR13" s="49" t="str"/>
-      <x:c r="AS13" s="50" t="str"/>
+      <x:c r="AS13" s="49" t="str"/>
+      <x:c r="AT13" s="49" t="str"/>
+      <x:c r="AU13" s="49" t="str"/>
+      <x:c r="AV13" s="50" t="str"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="48" t="str"/>
@@ -1936,7 +1990,10 @@
       <x:c r="AP14" s="49" t="str"/>
       <x:c r="AQ14" s="49" t="str"/>
       <x:c r="AR14" s="49" t="str"/>
-      <x:c r="AS14" s="50" t="str"/>
+      <x:c r="AS14" s="49" t="str"/>
+      <x:c r="AT14" s="49" t="str"/>
+      <x:c r="AU14" s="49" t="str"/>
+      <x:c r="AV14" s="50" t="str"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="48" t="str"/>
@@ -1983,7 +2040,10 @@
       <x:c r="AP15" s="49" t="str"/>
       <x:c r="AQ15" s="49" t="str"/>
       <x:c r="AR15" s="49" t="str"/>
-      <x:c r="AS15" s="50" t="str"/>
+      <x:c r="AS15" s="49" t="str"/>
+      <x:c r="AT15" s="49" t="str"/>
+      <x:c r="AU15" s="49" t="str"/>
+      <x:c r="AV15" s="50" t="str"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="48" t="str"/>
@@ -2030,7 +2090,10 @@
       <x:c r="AP16" s="49" t="str"/>
       <x:c r="AQ16" s="49" t="str"/>
       <x:c r="AR16" s="49" t="str"/>
-      <x:c r="AS16" s="50" t="str"/>
+      <x:c r="AS16" s="49" t="str"/>
+      <x:c r="AT16" s="49" t="str"/>
+      <x:c r="AU16" s="49" t="str"/>
+      <x:c r="AV16" s="50" t="str"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="48" t="str"/>
@@ -2077,7 +2140,10 @@
       <x:c r="AP17" s="49" t="str"/>
       <x:c r="AQ17" s="49" t="str"/>
       <x:c r="AR17" s="49" t="str"/>
-      <x:c r="AS17" s="50" t="str"/>
+      <x:c r="AS17" s="49" t="str"/>
+      <x:c r="AT17" s="49" t="str"/>
+      <x:c r="AU17" s="49" t="str"/>
+      <x:c r="AV17" s="50" t="str"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="48" t="str"/>
@@ -2124,7 +2190,10 @@
       <x:c r="AP18" s="49" t="str"/>
       <x:c r="AQ18" s="49" t="str"/>
       <x:c r="AR18" s="49" t="str"/>
-      <x:c r="AS18" s="50" t="str"/>
+      <x:c r="AS18" s="49" t="str"/>
+      <x:c r="AT18" s="49" t="str"/>
+      <x:c r="AU18" s="49" t="str"/>
+      <x:c r="AV18" s="50" t="str"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="48" t="str"/>
@@ -2171,7 +2240,10 @@
       <x:c r="AP19" s="49" t="str"/>
       <x:c r="AQ19" s="49" t="str"/>
       <x:c r="AR19" s="49" t="str"/>
-      <x:c r="AS19" s="50" t="str"/>
+      <x:c r="AS19" s="49" t="str"/>
+      <x:c r="AT19" s="49" t="str"/>
+      <x:c r="AU19" s="49" t="str"/>
+      <x:c r="AV19" s="50" t="str"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="48" t="str"/>
@@ -2218,7 +2290,10 @@
       <x:c r="AP20" s="49" t="str"/>
       <x:c r="AQ20" s="49" t="str"/>
       <x:c r="AR20" s="49" t="str"/>
-      <x:c r="AS20" s="50" t="str"/>
+      <x:c r="AS20" s="49" t="str"/>
+      <x:c r="AT20" s="49" t="str"/>
+      <x:c r="AU20" s="49" t="str"/>
+      <x:c r="AV20" s="50" t="str"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="48" t="str"/>
@@ -2265,7 +2340,10 @@
       <x:c r="AP21" s="49" t="str"/>
       <x:c r="AQ21" s="49" t="str"/>
       <x:c r="AR21" s="49" t="str"/>
-      <x:c r="AS21" s="50" t="str"/>
+      <x:c r="AS21" s="49" t="str"/>
+      <x:c r="AT21" s="49" t="str"/>
+      <x:c r="AU21" s="49" t="str"/>
+      <x:c r="AV21" s="50" t="str"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="48" t="str"/>
@@ -2312,7 +2390,10 @@
       <x:c r="AP22" s="49" t="str"/>
       <x:c r="AQ22" s="49" t="str"/>
       <x:c r="AR22" s="49" t="str"/>
-      <x:c r="AS22" s="50" t="str"/>
+      <x:c r="AS22" s="49" t="str"/>
+      <x:c r="AT22" s="49" t="str"/>
+      <x:c r="AU22" s="49" t="str"/>
+      <x:c r="AV22" s="50" t="str"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="48" t="str"/>
@@ -2359,7 +2440,10 @@
       <x:c r="AP23" s="49" t="str"/>
       <x:c r="AQ23" s="49" t="str"/>
       <x:c r="AR23" s="49" t="str"/>
-      <x:c r="AS23" s="50" t="str"/>
+      <x:c r="AS23" s="49" t="str"/>
+      <x:c r="AT23" s="49" t="str"/>
+      <x:c r="AU23" s="49" t="str"/>
+      <x:c r="AV23" s="50" t="str"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="48" t="str"/>
@@ -2406,7 +2490,10 @@
       <x:c r="AP24" s="49" t="str"/>
       <x:c r="AQ24" s="49" t="str"/>
       <x:c r="AR24" s="49" t="str"/>
-      <x:c r="AS24" s="50" t="str"/>
+      <x:c r="AS24" s="49" t="str"/>
+      <x:c r="AT24" s="49" t="str"/>
+      <x:c r="AU24" s="49" t="str"/>
+      <x:c r="AV24" s="50" t="str"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="48" t="str"/>
@@ -2453,7 +2540,10 @@
       <x:c r="AP25" s="49" t="str"/>
       <x:c r="AQ25" s="49" t="str"/>
       <x:c r="AR25" s="49" t="str"/>
-      <x:c r="AS25" s="50" t="str"/>
+      <x:c r="AS25" s="49" t="str"/>
+      <x:c r="AT25" s="49" t="str"/>
+      <x:c r="AU25" s="49" t="str"/>
+      <x:c r="AV25" s="50" t="str"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="48" t="str"/>
@@ -2500,7 +2590,10 @@
       <x:c r="AP26" s="49" t="str"/>
       <x:c r="AQ26" s="49" t="str"/>
       <x:c r="AR26" s="49" t="str"/>
-      <x:c r="AS26" s="50" t="str"/>
+      <x:c r="AS26" s="49" t="str"/>
+      <x:c r="AT26" s="49" t="str"/>
+      <x:c r="AU26" s="49" t="str"/>
+      <x:c r="AV26" s="50" t="str"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="48" t="str"/>
@@ -2547,7 +2640,10 @@
       <x:c r="AP27" s="49" t="str"/>
       <x:c r="AQ27" s="49" t="str"/>
       <x:c r="AR27" s="49" t="str"/>
-      <x:c r="AS27" s="50" t="str"/>
+      <x:c r="AS27" s="49" t="str"/>
+      <x:c r="AT27" s="49" t="str"/>
+      <x:c r="AU27" s="49" t="str"/>
+      <x:c r="AV27" s="50" t="str"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="48" t="str"/>
@@ -2594,7 +2690,10 @@
       <x:c r="AP28" s="49" t="str"/>
       <x:c r="AQ28" s="49" t="str"/>
       <x:c r="AR28" s="49" t="str"/>
-      <x:c r="AS28" s="50" t="str"/>
+      <x:c r="AS28" s="49" t="str"/>
+      <x:c r="AT28" s="49" t="str"/>
+      <x:c r="AU28" s="49" t="str"/>
+      <x:c r="AV28" s="50" t="str"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="48" t="str"/>
@@ -2641,7 +2740,10 @@
       <x:c r="AP29" s="49" t="str"/>
       <x:c r="AQ29" s="49" t="str"/>
       <x:c r="AR29" s="49" t="str"/>
-      <x:c r="AS29" s="50" t="str"/>
+      <x:c r="AS29" s="49" t="str"/>
+      <x:c r="AT29" s="49" t="str"/>
+      <x:c r="AU29" s="49" t="str"/>
+      <x:c r="AV29" s="50" t="str"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="48" t="str"/>
@@ -2688,7 +2790,10 @@
       <x:c r="AP30" s="49" t="str"/>
       <x:c r="AQ30" s="49" t="str"/>
       <x:c r="AR30" s="49" t="str"/>
-      <x:c r="AS30" s="50" t="str"/>
+      <x:c r="AS30" s="49" t="str"/>
+      <x:c r="AT30" s="49" t="str"/>
+      <x:c r="AU30" s="49" t="str"/>
+      <x:c r="AV30" s="50" t="str"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="48" t="str"/>
@@ -2735,7 +2840,10 @@
       <x:c r="AP31" s="49" t="str"/>
       <x:c r="AQ31" s="49" t="str"/>
       <x:c r="AR31" s="49" t="str"/>
-      <x:c r="AS31" s="50" t="str"/>
+      <x:c r="AS31" s="49" t="str"/>
+      <x:c r="AT31" s="49" t="str"/>
+      <x:c r="AU31" s="49" t="str"/>
+      <x:c r="AV31" s="50" t="str"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="48" t="str"/>
@@ -2782,7 +2890,10 @@
       <x:c r="AP32" s="49" t="str"/>
       <x:c r="AQ32" s="49" t="str"/>
       <x:c r="AR32" s="49" t="str"/>
-      <x:c r="AS32" s="50" t="str"/>
+      <x:c r="AS32" s="49" t="str"/>
+      <x:c r="AT32" s="49" t="str"/>
+      <x:c r="AU32" s="49" t="str"/>
+      <x:c r="AV32" s="50" t="str"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="48" t="str"/>
@@ -2829,7 +2940,10 @@
       <x:c r="AP33" s="49" t="str"/>
       <x:c r="AQ33" s="49" t="str"/>
       <x:c r="AR33" s="49" t="str"/>
-      <x:c r="AS33" s="50" t="str"/>
+      <x:c r="AS33" s="49" t="str"/>
+      <x:c r="AT33" s="49" t="str"/>
+      <x:c r="AU33" s="49" t="str"/>
+      <x:c r="AV33" s="50" t="str"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="48" t="str"/>
@@ -2876,7 +2990,10 @@
       <x:c r="AP34" s="49" t="str"/>
       <x:c r="AQ34" s="49" t="str"/>
       <x:c r="AR34" s="49" t="str"/>
-      <x:c r="AS34" s="50" t="str"/>
+      <x:c r="AS34" s="49" t="str"/>
+      <x:c r="AT34" s="49" t="str"/>
+      <x:c r="AU34" s="49" t="str"/>
+      <x:c r="AV34" s="50" t="str"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="48" t="str"/>
@@ -2923,7 +3040,10 @@
       <x:c r="AP35" s="49" t="str"/>
       <x:c r="AQ35" s="49" t="str"/>
       <x:c r="AR35" s="49" t="str"/>
-      <x:c r="AS35" s="50" t="str"/>
+      <x:c r="AS35" s="49" t="str"/>
+      <x:c r="AT35" s="49" t="str"/>
+      <x:c r="AU35" s="49" t="str"/>
+      <x:c r="AV35" s="50" t="str"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="48" t="str"/>
@@ -2970,7 +3090,10 @@
       <x:c r="AP36" s="49" t="str"/>
       <x:c r="AQ36" s="49" t="str"/>
       <x:c r="AR36" s="49" t="str"/>
-      <x:c r="AS36" s="50" t="str"/>
+      <x:c r="AS36" s="49" t="str"/>
+      <x:c r="AT36" s="49" t="str"/>
+      <x:c r="AU36" s="49" t="str"/>
+      <x:c r="AV36" s="50" t="str"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="48" t="str"/>
@@ -3017,7 +3140,10 @@
       <x:c r="AP37" s="49" t="str"/>
       <x:c r="AQ37" s="49" t="str"/>
       <x:c r="AR37" s="49" t="str"/>
-      <x:c r="AS37" s="50" t="str"/>
+      <x:c r="AS37" s="49" t="str"/>
+      <x:c r="AT37" s="49" t="str"/>
+      <x:c r="AU37" s="49" t="str"/>
+      <x:c r="AV37" s="50" t="str"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="48" t="str"/>
@@ -3064,7 +3190,10 @@
       <x:c r="AP38" s="49" t="str"/>
       <x:c r="AQ38" s="49" t="str"/>
       <x:c r="AR38" s="49" t="str"/>
-      <x:c r="AS38" s="50" t="str"/>
+      <x:c r="AS38" s="49" t="str"/>
+      <x:c r="AT38" s="49" t="str"/>
+      <x:c r="AU38" s="49" t="str"/>
+      <x:c r="AV38" s="50" t="str"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="48" t="str"/>
@@ -3111,7 +3240,10 @@
       <x:c r="AP39" s="49" t="str"/>
       <x:c r="AQ39" s="49" t="str"/>
       <x:c r="AR39" s="49" t="str"/>
-      <x:c r="AS39" s="50" t="str"/>
+      <x:c r="AS39" s="49" t="str"/>
+      <x:c r="AT39" s="49" t="str"/>
+      <x:c r="AU39" s="49" t="str"/>
+      <x:c r="AV39" s="50" t="str"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="48" t="str"/>
@@ -3158,7 +3290,10 @@
       <x:c r="AP40" s="49" t="str"/>
       <x:c r="AQ40" s="49" t="str"/>
       <x:c r="AR40" s="49" t="str"/>
-      <x:c r="AS40" s="50" t="str"/>
+      <x:c r="AS40" s="49" t="str"/>
+      <x:c r="AT40" s="49" t="str"/>
+      <x:c r="AU40" s="49" t="str"/>
+      <x:c r="AV40" s="50" t="str"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="48" t="str"/>
@@ -3205,7 +3340,10 @@
       <x:c r="AP41" s="49" t="str"/>
       <x:c r="AQ41" s="49" t="str"/>
       <x:c r="AR41" s="49" t="str"/>
-      <x:c r="AS41" s="50" t="str"/>
+      <x:c r="AS41" s="49" t="str"/>
+      <x:c r="AT41" s="49" t="str"/>
+      <x:c r="AU41" s="49" t="str"/>
+      <x:c r="AV41" s="50" t="str"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="48" t="str"/>
@@ -3252,7 +3390,10 @@
       <x:c r="AP42" s="49" t="str"/>
       <x:c r="AQ42" s="49" t="str"/>
       <x:c r="AR42" s="49" t="str"/>
-      <x:c r="AS42" s="50" t="str"/>
+      <x:c r="AS42" s="49" t="str"/>
+      <x:c r="AT42" s="49" t="str"/>
+      <x:c r="AU42" s="49" t="str"/>
+      <x:c r="AV42" s="50" t="str"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="48" t="str"/>
@@ -3299,7 +3440,10 @@
       <x:c r="AP43" s="49" t="str"/>
       <x:c r="AQ43" s="49" t="str"/>
       <x:c r="AR43" s="49" t="str"/>
-      <x:c r="AS43" s="50" t="str"/>
+      <x:c r="AS43" s="49" t="str"/>
+      <x:c r="AT43" s="49" t="str"/>
+      <x:c r="AU43" s="49" t="str"/>
+      <x:c r="AV43" s="50" t="str"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="48" t="str"/>
@@ -3346,7 +3490,10 @@
       <x:c r="AP44" s="49" t="str"/>
       <x:c r="AQ44" s="49" t="str"/>
       <x:c r="AR44" s="49" t="str"/>
-      <x:c r="AS44" s="50" t="str"/>
+      <x:c r="AS44" s="49" t="str"/>
+      <x:c r="AT44" s="49" t="str"/>
+      <x:c r="AU44" s="49" t="str"/>
+      <x:c r="AV44" s="50" t="str"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="48" t="str"/>
@@ -3393,7 +3540,10 @@
       <x:c r="AP45" s="49" t="str"/>
       <x:c r="AQ45" s="49" t="str"/>
       <x:c r="AR45" s="49" t="str"/>
-      <x:c r="AS45" s="50" t="str"/>
+      <x:c r="AS45" s="49" t="str"/>
+      <x:c r="AT45" s="49" t="str"/>
+      <x:c r="AU45" s="49" t="str"/>
+      <x:c r="AV45" s="50" t="str"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="48" t="str"/>
@@ -3440,7 +3590,10 @@
       <x:c r="AP46" s="49" t="str"/>
       <x:c r="AQ46" s="49" t="str"/>
       <x:c r="AR46" s="49" t="str"/>
-      <x:c r="AS46" s="50" t="str"/>
+      <x:c r="AS46" s="49" t="str"/>
+      <x:c r="AT46" s="49" t="str"/>
+      <x:c r="AU46" s="49" t="str"/>
+      <x:c r="AV46" s="50" t="str"/>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="48" t="str"/>
@@ -3487,7 +3640,10 @@
       <x:c r="AP47" s="49" t="str"/>
       <x:c r="AQ47" s="49" t="str"/>
       <x:c r="AR47" s="49" t="str"/>
-      <x:c r="AS47" s="50" t="str"/>
+      <x:c r="AS47" s="49" t="str"/>
+      <x:c r="AT47" s="49" t="str"/>
+      <x:c r="AU47" s="49" t="str"/>
+      <x:c r="AV47" s="50" t="str"/>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="48" t="str"/>
@@ -3534,7 +3690,10 @@
       <x:c r="AP48" s="49" t="str"/>
       <x:c r="AQ48" s="49" t="str"/>
       <x:c r="AR48" s="49" t="str"/>
-      <x:c r="AS48" s="50" t="str"/>
+      <x:c r="AS48" s="49" t="str"/>
+      <x:c r="AT48" s="49" t="str"/>
+      <x:c r="AU48" s="49" t="str"/>
+      <x:c r="AV48" s="50" t="str"/>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="48" t="str"/>
@@ -3581,7 +3740,10 @@
       <x:c r="AP49" s="49" t="str"/>
       <x:c r="AQ49" s="49" t="str"/>
       <x:c r="AR49" s="49" t="str"/>
-      <x:c r="AS49" s="50" t="str"/>
+      <x:c r="AS49" s="49" t="str"/>
+      <x:c r="AT49" s="49" t="str"/>
+      <x:c r="AU49" s="49" t="str"/>
+      <x:c r="AV49" s="50" t="str"/>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="48" t="str"/>
@@ -3628,7 +3790,10 @@
       <x:c r="AP50" s="49" t="str"/>
       <x:c r="AQ50" s="49" t="str"/>
       <x:c r="AR50" s="49" t="str"/>
-      <x:c r="AS50" s="50" t="str"/>
+      <x:c r="AS50" s="49" t="str"/>
+      <x:c r="AT50" s="49" t="str"/>
+      <x:c r="AU50" s="49" t="str"/>
+      <x:c r="AV50" s="50" t="str"/>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="48" t="str"/>
@@ -3675,7 +3840,10 @@
       <x:c r="AP51" s="49" t="str"/>
       <x:c r="AQ51" s="49" t="str"/>
       <x:c r="AR51" s="49" t="str"/>
-      <x:c r="AS51" s="50" t="str"/>
+      <x:c r="AS51" s="49" t="str"/>
+      <x:c r="AT51" s="49" t="str"/>
+      <x:c r="AU51" s="49" t="str"/>
+      <x:c r="AV51" s="50" t="str"/>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="48" t="str"/>
@@ -3722,7 +3890,10 @@
       <x:c r="AP52" s="49" t="str"/>
       <x:c r="AQ52" s="49" t="str"/>
       <x:c r="AR52" s="49" t="str"/>
-      <x:c r="AS52" s="50" t="str"/>
+      <x:c r="AS52" s="49" t="str"/>
+      <x:c r="AT52" s="49" t="str"/>
+      <x:c r="AU52" s="49" t="str"/>
+      <x:c r="AV52" s="50" t="str"/>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="48" t="str"/>
@@ -3769,7 +3940,10 @@
       <x:c r="AP53" s="49" t="str"/>
       <x:c r="AQ53" s="49" t="str"/>
       <x:c r="AR53" s="49" t="str"/>
-      <x:c r="AS53" s="50" t="str"/>
+      <x:c r="AS53" s="49" t="str"/>
+      <x:c r="AT53" s="49" t="str"/>
+      <x:c r="AU53" s="49" t="str"/>
+      <x:c r="AV53" s="50" t="str"/>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="48" t="str"/>
@@ -3816,7 +3990,10 @@
       <x:c r="AP54" s="49" t="str"/>
       <x:c r="AQ54" s="49" t="str"/>
       <x:c r="AR54" s="49" t="str"/>
-      <x:c r="AS54" s="50" t="str"/>
+      <x:c r="AS54" s="49" t="str"/>
+      <x:c r="AT54" s="49" t="str"/>
+      <x:c r="AU54" s="49" t="str"/>
+      <x:c r="AV54" s="50" t="str"/>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="48" t="str"/>
@@ -3863,7 +4040,10 @@
       <x:c r="AP55" s="49" t="str"/>
       <x:c r="AQ55" s="49" t="str"/>
       <x:c r="AR55" s="49" t="str"/>
-      <x:c r="AS55" s="50" t="str"/>
+      <x:c r="AS55" s="49" t="str"/>
+      <x:c r="AT55" s="49" t="str"/>
+      <x:c r="AU55" s="49" t="str"/>
+      <x:c r="AV55" s="50" t="str"/>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="48" t="str"/>
@@ -3910,7 +4090,10 @@
       <x:c r="AP56" s="49" t="str"/>
       <x:c r="AQ56" s="49" t="str"/>
       <x:c r="AR56" s="49" t="str"/>
-      <x:c r="AS56" s="50" t="str"/>
+      <x:c r="AS56" s="49" t="str"/>
+      <x:c r="AT56" s="49" t="str"/>
+      <x:c r="AU56" s="49" t="str"/>
+      <x:c r="AV56" s="50" t="str"/>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="48" t="str"/>
@@ -3957,7 +4140,10 @@
       <x:c r="AP57" s="49" t="str"/>
       <x:c r="AQ57" s="49" t="str"/>
       <x:c r="AR57" s="49" t="str"/>
-      <x:c r="AS57" s="50" t="str"/>
+      <x:c r="AS57" s="49" t="str"/>
+      <x:c r="AT57" s="49" t="str"/>
+      <x:c r="AU57" s="49" t="str"/>
+      <x:c r="AV57" s="50" t="str"/>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="48" t="str"/>
@@ -4004,7 +4190,10 @@
       <x:c r="AP58" s="49" t="str"/>
       <x:c r="AQ58" s="49" t="str"/>
       <x:c r="AR58" s="49" t="str"/>
-      <x:c r="AS58" s="50" t="str"/>
+      <x:c r="AS58" s="49" t="str"/>
+      <x:c r="AT58" s="49" t="str"/>
+      <x:c r="AU58" s="49" t="str"/>
+      <x:c r="AV58" s="50" t="str"/>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="48" t="str"/>
@@ -4051,7 +4240,10 @@
       <x:c r="AP59" s="49" t="str"/>
       <x:c r="AQ59" s="49" t="str"/>
       <x:c r="AR59" s="49" t="str"/>
-      <x:c r="AS59" s="50" t="str"/>
+      <x:c r="AS59" s="49" t="str"/>
+      <x:c r="AT59" s="49" t="str"/>
+      <x:c r="AU59" s="49" t="str"/>
+      <x:c r="AV59" s="50" t="str"/>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="48" t="str"/>
@@ -4098,7 +4290,10 @@
       <x:c r="AP60" s="49" t="str"/>
       <x:c r="AQ60" s="49" t="str"/>
       <x:c r="AR60" s="49" t="str"/>
-      <x:c r="AS60" s="50" t="str"/>
+      <x:c r="AS60" s="49" t="str"/>
+      <x:c r="AT60" s="49" t="str"/>
+      <x:c r="AU60" s="49" t="str"/>
+      <x:c r="AV60" s="50" t="str"/>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="48" t="str"/>
@@ -4145,7 +4340,10 @@
       <x:c r="AP61" s="49" t="str"/>
       <x:c r="AQ61" s="49" t="str"/>
       <x:c r="AR61" s="49" t="str"/>
-      <x:c r="AS61" s="50" t="str"/>
+      <x:c r="AS61" s="49" t="str"/>
+      <x:c r="AT61" s="49" t="str"/>
+      <x:c r="AU61" s="49" t="str"/>
+      <x:c r="AV61" s="50" t="str"/>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="48" t="str"/>
@@ -4192,7 +4390,10 @@
       <x:c r="AP62" s="49" t="str"/>
       <x:c r="AQ62" s="49" t="str"/>
       <x:c r="AR62" s="49" t="str"/>
-      <x:c r="AS62" s="50" t="str"/>
+      <x:c r="AS62" s="49" t="str"/>
+      <x:c r="AT62" s="49" t="str"/>
+      <x:c r="AU62" s="49" t="str"/>
+      <x:c r="AV62" s="50" t="str"/>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="48" t="str"/>
@@ -4239,7 +4440,10 @@
       <x:c r="AP63" s="49" t="str"/>
       <x:c r="AQ63" s="49" t="str"/>
       <x:c r="AR63" s="49" t="str"/>
-      <x:c r="AS63" s="50" t="str"/>
+      <x:c r="AS63" s="49" t="str"/>
+      <x:c r="AT63" s="49" t="str"/>
+      <x:c r="AU63" s="49" t="str"/>
+      <x:c r="AV63" s="50" t="str"/>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="48" t="str"/>
@@ -4286,7 +4490,10 @@
       <x:c r="AP64" s="49" t="str"/>
       <x:c r="AQ64" s="49" t="str"/>
       <x:c r="AR64" s="49" t="str"/>
-      <x:c r="AS64" s="50" t="str"/>
+      <x:c r="AS64" s="49" t="str"/>
+      <x:c r="AT64" s="49" t="str"/>
+      <x:c r="AU64" s="49" t="str"/>
+      <x:c r="AV64" s="50" t="str"/>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="48" t="str"/>
@@ -4333,7 +4540,10 @@
       <x:c r="AP65" s="49" t="str"/>
       <x:c r="AQ65" s="49" t="str"/>
       <x:c r="AR65" s="49" t="str"/>
-      <x:c r="AS65" s="50" t="str"/>
+      <x:c r="AS65" s="49" t="str"/>
+      <x:c r="AT65" s="49" t="str"/>
+      <x:c r="AU65" s="49" t="str"/>
+      <x:c r="AV65" s="50" t="str"/>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="48" t="str"/>
@@ -4380,7 +4590,10 @@
       <x:c r="AP66" s="49" t="str"/>
       <x:c r="AQ66" s="49" t="str"/>
       <x:c r="AR66" s="49" t="str"/>
-      <x:c r="AS66" s="50" t="str"/>
+      <x:c r="AS66" s="49" t="str"/>
+      <x:c r="AT66" s="49" t="str"/>
+      <x:c r="AU66" s="49" t="str"/>
+      <x:c r="AV66" s="50" t="str"/>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="48" t="str"/>
@@ -4427,7 +4640,10 @@
       <x:c r="AP67" s="49" t="str"/>
       <x:c r="AQ67" s="49" t="str"/>
       <x:c r="AR67" s="49" t="str"/>
-      <x:c r="AS67" s="50" t="str"/>
+      <x:c r="AS67" s="49" t="str"/>
+      <x:c r="AT67" s="49" t="str"/>
+      <x:c r="AU67" s="49" t="str"/>
+      <x:c r="AV67" s="50" t="str"/>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="48" t="str"/>
@@ -4474,7 +4690,10 @@
       <x:c r="AP68" s="49" t="str"/>
       <x:c r="AQ68" s="49" t="str"/>
       <x:c r="AR68" s="49" t="str"/>
-      <x:c r="AS68" s="50" t="str"/>
+      <x:c r="AS68" s="49" t="str"/>
+      <x:c r="AT68" s="49" t="str"/>
+      <x:c r="AU68" s="49" t="str"/>
+      <x:c r="AV68" s="50" t="str"/>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="48" t="str"/>
@@ -4521,7 +4740,10 @@
       <x:c r="AP69" s="49" t="str"/>
       <x:c r="AQ69" s="49" t="str"/>
       <x:c r="AR69" s="49" t="str"/>
-      <x:c r="AS69" s="50" t="str"/>
+      <x:c r="AS69" s="49" t="str"/>
+      <x:c r="AT69" s="49" t="str"/>
+      <x:c r="AU69" s="49" t="str"/>
+      <x:c r="AV69" s="50" t="str"/>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="48" t="str"/>
@@ -4568,7 +4790,10 @@
       <x:c r="AP70" s="49" t="str"/>
       <x:c r="AQ70" s="49" t="str"/>
       <x:c r="AR70" s="49" t="str"/>
-      <x:c r="AS70" s="50" t="str"/>
+      <x:c r="AS70" s="49" t="str"/>
+      <x:c r="AT70" s="49" t="str"/>
+      <x:c r="AU70" s="49" t="str"/>
+      <x:c r="AV70" s="50" t="str"/>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="48" t="str"/>
@@ -4615,7 +4840,10 @@
       <x:c r="AP71" s="49" t="str"/>
       <x:c r="AQ71" s="49" t="str"/>
       <x:c r="AR71" s="49" t="str"/>
-      <x:c r="AS71" s="50" t="str"/>
+      <x:c r="AS71" s="49" t="str"/>
+      <x:c r="AT71" s="49" t="str"/>
+      <x:c r="AU71" s="49" t="str"/>
+      <x:c r="AV71" s="50" t="str"/>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="48" t="str"/>
@@ -4662,7 +4890,10 @@
       <x:c r="AP72" s="49" t="str"/>
       <x:c r="AQ72" s="49" t="str"/>
       <x:c r="AR72" s="49" t="str"/>
-      <x:c r="AS72" s="50" t="str"/>
+      <x:c r="AS72" s="49" t="str"/>
+      <x:c r="AT72" s="49" t="str"/>
+      <x:c r="AU72" s="49" t="str"/>
+      <x:c r="AV72" s="50" t="str"/>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="48" t="str"/>
@@ -4709,7 +4940,10 @@
       <x:c r="AP73" s="49" t="str"/>
       <x:c r="AQ73" s="49" t="str"/>
       <x:c r="AR73" s="49" t="str"/>
-      <x:c r="AS73" s="50" t="str"/>
+      <x:c r="AS73" s="49" t="str"/>
+      <x:c r="AT73" s="49" t="str"/>
+      <x:c r="AU73" s="49" t="str"/>
+      <x:c r="AV73" s="50" t="str"/>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="48" t="str"/>
@@ -4756,7 +4990,10 @@
       <x:c r="AP74" s="49" t="str"/>
       <x:c r="AQ74" s="49" t="str"/>
       <x:c r="AR74" s="49" t="str"/>
-      <x:c r="AS74" s="50" t="str"/>
+      <x:c r="AS74" s="49" t="str"/>
+      <x:c r="AT74" s="49" t="str"/>
+      <x:c r="AU74" s="49" t="str"/>
+      <x:c r="AV74" s="50" t="str"/>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="48" t="str"/>
@@ -4803,7 +5040,10 @@
       <x:c r="AP75" s="49" t="str"/>
       <x:c r="AQ75" s="49" t="str"/>
       <x:c r="AR75" s="49" t="str"/>
-      <x:c r="AS75" s="50" t="str"/>
+      <x:c r="AS75" s="49" t="str"/>
+      <x:c r="AT75" s="49" t="str"/>
+      <x:c r="AU75" s="49" t="str"/>
+      <x:c r="AV75" s="50" t="str"/>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="48" t="str"/>
@@ -4850,7 +5090,10 @@
       <x:c r="AP76" s="49" t="str"/>
       <x:c r="AQ76" s="49" t="str"/>
       <x:c r="AR76" s="49" t="str"/>
-      <x:c r="AS76" s="50" t="str"/>
+      <x:c r="AS76" s="49" t="str"/>
+      <x:c r="AT76" s="49" t="str"/>
+      <x:c r="AU76" s="49" t="str"/>
+      <x:c r="AV76" s="50" t="str"/>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="48" t="str"/>
@@ -4897,7 +5140,10 @@
       <x:c r="AP77" s="49" t="str"/>
       <x:c r="AQ77" s="49" t="str"/>
       <x:c r="AR77" s="49" t="str"/>
-      <x:c r="AS77" s="50" t="str"/>
+      <x:c r="AS77" s="49" t="str"/>
+      <x:c r="AT77" s="49" t="str"/>
+      <x:c r="AU77" s="49" t="str"/>
+      <x:c r="AV77" s="50" t="str"/>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="48" t="str"/>
@@ -4944,7 +5190,10 @@
       <x:c r="AP78" s="49" t="str"/>
       <x:c r="AQ78" s="49" t="str"/>
       <x:c r="AR78" s="49" t="str"/>
-      <x:c r="AS78" s="50" t="str"/>
+      <x:c r="AS78" s="49" t="str"/>
+      <x:c r="AT78" s="49" t="str"/>
+      <x:c r="AU78" s="49" t="str"/>
+      <x:c r="AV78" s="50" t="str"/>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="48" t="str"/>
@@ -4991,7 +5240,10 @@
       <x:c r="AP79" s="49" t="str"/>
       <x:c r="AQ79" s="49" t="str"/>
       <x:c r="AR79" s="49" t="str"/>
-      <x:c r="AS79" s="50" t="str"/>
+      <x:c r="AS79" s="49" t="str"/>
+      <x:c r="AT79" s="49" t="str"/>
+      <x:c r="AU79" s="49" t="str"/>
+      <x:c r="AV79" s="50" t="str"/>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="48" t="str"/>
@@ -5038,7 +5290,10 @@
       <x:c r="AP80" s="49" t="str"/>
       <x:c r="AQ80" s="49" t="str"/>
       <x:c r="AR80" s="49" t="str"/>
-      <x:c r="AS80" s="50" t="str"/>
+      <x:c r="AS80" s="49" t="str"/>
+      <x:c r="AT80" s="49" t="str"/>
+      <x:c r="AU80" s="49" t="str"/>
+      <x:c r="AV80" s="50" t="str"/>
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="48" t="str"/>
@@ -5085,7 +5340,10 @@
       <x:c r="AP81" s="49" t="str"/>
       <x:c r="AQ81" s="49" t="str"/>
       <x:c r="AR81" s="49" t="str"/>
-      <x:c r="AS81" s="50" t="str"/>
+      <x:c r="AS81" s="49" t="str"/>
+      <x:c r="AT81" s="49" t="str"/>
+      <x:c r="AU81" s="49" t="str"/>
+      <x:c r="AV81" s="50" t="str"/>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="48" t="str"/>
@@ -5132,7 +5390,10 @@
       <x:c r="AP82" s="49" t="str"/>
       <x:c r="AQ82" s="49" t="str"/>
       <x:c r="AR82" s="49" t="str"/>
-      <x:c r="AS82" s="50" t="str"/>
+      <x:c r="AS82" s="49" t="str"/>
+      <x:c r="AT82" s="49" t="str"/>
+      <x:c r="AU82" s="49" t="str"/>
+      <x:c r="AV82" s="50" t="str"/>
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="48" t="str"/>
@@ -5179,7 +5440,10 @@
       <x:c r="AP83" s="49" t="str"/>
       <x:c r="AQ83" s="49" t="str"/>
       <x:c r="AR83" s="49" t="str"/>
-      <x:c r="AS83" s="50" t="str"/>
+      <x:c r="AS83" s="49" t="str"/>
+      <x:c r="AT83" s="49" t="str"/>
+      <x:c r="AU83" s="49" t="str"/>
+      <x:c r="AV83" s="50" t="str"/>
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="48" t="str"/>
@@ -5226,7 +5490,10 @@
       <x:c r="AP84" s="49" t="str"/>
       <x:c r="AQ84" s="49" t="str"/>
       <x:c r="AR84" s="49" t="str"/>
-      <x:c r="AS84" s="50" t="str"/>
+      <x:c r="AS84" s="49" t="str"/>
+      <x:c r="AT84" s="49" t="str"/>
+      <x:c r="AU84" s="49" t="str"/>
+      <x:c r="AV84" s="50" t="str"/>
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="48" t="str"/>
@@ -5273,7 +5540,10 @@
       <x:c r="AP85" s="49" t="str"/>
       <x:c r="AQ85" s="49" t="str"/>
       <x:c r="AR85" s="49" t="str"/>
-      <x:c r="AS85" s="50" t="str"/>
+      <x:c r="AS85" s="49" t="str"/>
+      <x:c r="AT85" s="49" t="str"/>
+      <x:c r="AU85" s="49" t="str"/>
+      <x:c r="AV85" s="50" t="str"/>
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="48" t="str"/>
@@ -5320,7 +5590,10 @@
       <x:c r="AP86" s="49" t="str"/>
       <x:c r="AQ86" s="49" t="str"/>
       <x:c r="AR86" s="49" t="str"/>
-      <x:c r="AS86" s="50" t="str"/>
+      <x:c r="AS86" s="49" t="str"/>
+      <x:c r="AT86" s="49" t="str"/>
+      <x:c r="AU86" s="49" t="str"/>
+      <x:c r="AV86" s="50" t="str"/>
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="48" t="str"/>
@@ -5367,7 +5640,10 @@
       <x:c r="AP87" s="49" t="str"/>
       <x:c r="AQ87" s="49" t="str"/>
       <x:c r="AR87" s="49" t="str"/>
-      <x:c r="AS87" s="50" t="str"/>
+      <x:c r="AS87" s="49" t="str"/>
+      <x:c r="AT87" s="49" t="str"/>
+      <x:c r="AU87" s="49" t="str"/>
+      <x:c r="AV87" s="50" t="str"/>
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="48" t="str"/>
@@ -5414,7 +5690,10 @@
       <x:c r="AP88" s="49" t="str"/>
       <x:c r="AQ88" s="49" t="str"/>
       <x:c r="AR88" s="49" t="str"/>
-      <x:c r="AS88" s="50" t="str"/>
+      <x:c r="AS88" s="49" t="str"/>
+      <x:c r="AT88" s="49" t="str"/>
+      <x:c r="AU88" s="49" t="str"/>
+      <x:c r="AV88" s="50" t="str"/>
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="48" t="str"/>
@@ -5461,7 +5740,10 @@
       <x:c r="AP89" s="49" t="str"/>
       <x:c r="AQ89" s="49" t="str"/>
       <x:c r="AR89" s="49" t="str"/>
-      <x:c r="AS89" s="50" t="str"/>
+      <x:c r="AS89" s="49" t="str"/>
+      <x:c r="AT89" s="49" t="str"/>
+      <x:c r="AU89" s="49" t="str"/>
+      <x:c r="AV89" s="50" t="str"/>
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="48" t="str"/>
@@ -5508,7 +5790,10 @@
       <x:c r="AP90" s="49" t="str"/>
       <x:c r="AQ90" s="49" t="str"/>
       <x:c r="AR90" s="49" t="str"/>
-      <x:c r="AS90" s="50" t="str"/>
+      <x:c r="AS90" s="49" t="str"/>
+      <x:c r="AT90" s="49" t="str"/>
+      <x:c r="AU90" s="49" t="str"/>
+      <x:c r="AV90" s="50" t="str"/>
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="48" t="str"/>
@@ -5555,7 +5840,10 @@
       <x:c r="AP91" s="49" t="str"/>
       <x:c r="AQ91" s="49" t="str"/>
       <x:c r="AR91" s="49" t="str"/>
-      <x:c r="AS91" s="50" t="str"/>
+      <x:c r="AS91" s="49" t="str"/>
+      <x:c r="AT91" s="49" t="str"/>
+      <x:c r="AU91" s="49" t="str"/>
+      <x:c r="AV91" s="50" t="str"/>
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="48" t="str"/>
@@ -5602,7 +5890,10 @@
       <x:c r="AP92" s="49" t="str"/>
       <x:c r="AQ92" s="49" t="str"/>
       <x:c r="AR92" s="49" t="str"/>
-      <x:c r="AS92" s="50" t="str"/>
+      <x:c r="AS92" s="49" t="str"/>
+      <x:c r="AT92" s="49" t="str"/>
+      <x:c r="AU92" s="49" t="str"/>
+      <x:c r="AV92" s="50" t="str"/>
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="48" t="str"/>
@@ -5649,7 +5940,10 @@
       <x:c r="AP93" s="49" t="str"/>
       <x:c r="AQ93" s="49" t="str"/>
       <x:c r="AR93" s="49" t="str"/>
-      <x:c r="AS93" s="50" t="str"/>
+      <x:c r="AS93" s="49" t="str"/>
+      <x:c r="AT93" s="49" t="str"/>
+      <x:c r="AU93" s="49" t="str"/>
+      <x:c r="AV93" s="50" t="str"/>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="48" t="str"/>
@@ -5696,7 +5990,10 @@
       <x:c r="AP94" s="49" t="str"/>
       <x:c r="AQ94" s="49" t="str"/>
       <x:c r="AR94" s="49" t="str"/>
-      <x:c r="AS94" s="50" t="str"/>
+      <x:c r="AS94" s="49" t="str"/>
+      <x:c r="AT94" s="49" t="str"/>
+      <x:c r="AU94" s="49" t="str"/>
+      <x:c r="AV94" s="50" t="str"/>
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="48" t="str"/>
@@ -5743,7 +6040,10 @@
       <x:c r="AP95" s="49" t="str"/>
       <x:c r="AQ95" s="49" t="str"/>
       <x:c r="AR95" s="49" t="str"/>
-      <x:c r="AS95" s="50" t="str"/>
+      <x:c r="AS95" s="49" t="str"/>
+      <x:c r="AT95" s="49" t="str"/>
+      <x:c r="AU95" s="49" t="str"/>
+      <x:c r="AV95" s="50" t="str"/>
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="48" t="str"/>
@@ -5790,7 +6090,10 @@
       <x:c r="AP96" s="49" t="str"/>
       <x:c r="AQ96" s="49" t="str"/>
       <x:c r="AR96" s="49" t="str"/>
-      <x:c r="AS96" s="50" t="str"/>
+      <x:c r="AS96" s="49" t="str"/>
+      <x:c r="AT96" s="49" t="str"/>
+      <x:c r="AU96" s="49" t="str"/>
+      <x:c r="AV96" s="50" t="str"/>
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="48" t="str"/>
@@ -5837,7 +6140,10 @@
       <x:c r="AP97" s="49" t="str"/>
       <x:c r="AQ97" s="49" t="str"/>
       <x:c r="AR97" s="49" t="str"/>
-      <x:c r="AS97" s="50" t="str"/>
+      <x:c r="AS97" s="49" t="str"/>
+      <x:c r="AT97" s="49" t="str"/>
+      <x:c r="AU97" s="49" t="str"/>
+      <x:c r="AV97" s="50" t="str"/>
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="48" t="str"/>
@@ -5884,7 +6190,10 @@
       <x:c r="AP98" s="49" t="str"/>
       <x:c r="AQ98" s="49" t="str"/>
       <x:c r="AR98" s="49" t="str"/>
-      <x:c r="AS98" s="50" t="str"/>
+      <x:c r="AS98" s="49" t="str"/>
+      <x:c r="AT98" s="49" t="str"/>
+      <x:c r="AU98" s="49" t="str"/>
+      <x:c r="AV98" s="50" t="str"/>
     </x:row>
     <x:row r="99">
       <x:c r="A99" s="48" t="str"/>
@@ -5931,7 +6240,10 @@
       <x:c r="AP99" s="49" t="str"/>
       <x:c r="AQ99" s="49" t="str"/>
       <x:c r="AR99" s="49" t="str"/>
-      <x:c r="AS99" s="50" t="str"/>
+      <x:c r="AS99" s="49" t="str"/>
+      <x:c r="AT99" s="49" t="str"/>
+      <x:c r="AU99" s="49" t="str"/>
+      <x:c r="AV99" s="50" t="str"/>
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="48" t="str"/>
@@ -5978,7 +6290,10 @@
       <x:c r="AP100" s="49" t="str"/>
       <x:c r="AQ100" s="49" t="str"/>
       <x:c r="AR100" s="49" t="str"/>
-      <x:c r="AS100" s="50" t="str"/>
+      <x:c r="AS100" s="49" t="str"/>
+      <x:c r="AT100" s="49" t="str"/>
+      <x:c r="AU100" s="49" t="str"/>
+      <x:c r="AV100" s="50" t="str"/>
     </x:row>
     <x:row r="101">
       <x:c r="A101" s="48" t="str"/>
@@ -6025,7 +6340,10 @@
       <x:c r="AP101" s="49" t="str"/>
       <x:c r="AQ101" s="49" t="str"/>
       <x:c r="AR101" s="49" t="str"/>
-      <x:c r="AS101" s="50" t="str"/>
+      <x:c r="AS101" s="49" t="str"/>
+      <x:c r="AT101" s="49" t="str"/>
+      <x:c r="AU101" s="49" t="str"/>
+      <x:c r="AV101" s="50" t="str"/>
     </x:row>
     <x:row r="102">
       <x:c r="A102" s="48" t="str"/>
@@ -6072,7 +6390,10 @@
       <x:c r="AP102" s="49" t="str"/>
       <x:c r="AQ102" s="49" t="str"/>
       <x:c r="AR102" s="49" t="str"/>
-      <x:c r="AS102" s="50" t="str"/>
+      <x:c r="AS102" s="49" t="str"/>
+      <x:c r="AT102" s="49" t="str"/>
+      <x:c r="AU102" s="49" t="str"/>
+      <x:c r="AV102" s="50" t="str"/>
     </x:row>
     <x:row r="103">
       <x:c r="A103" s="51" t="str"/>
@@ -6119,16 +6440,19 @@
       <x:c r="AP103" s="52" t="str"/>
       <x:c r="AQ103" s="52" t="str"/>
       <x:c r="AR103" s="52" t="str"/>
-      <x:c r="AS103" s="53" t="str"/>
+      <x:c r="AS103" s="52" t="str"/>
+      <x:c r="AT103" s="52" t="str"/>
+      <x:c r="AU103" s="52" t="str"/>
+      <x:c r="AV103" s="53" t="str"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:AS1"/>
-    <x:mergeCell ref="A2:AS2"/>
+    <x:mergeCell ref="A1:AV1"/>
+    <x:mergeCell ref="A2:AV2"/>
   </x:mergeCells>
-  <x:dataValidations count="17">
+  <x:dataValidations count="20">
     <x:dataValidation type="list" sqref="B4:B103">
-      <x:formula1>Lists!$A$4:$A$9</x:formula1>
+      <x:formula1>Lists!$A$4:$A$10</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="I4:I103">
       <x:formula1>Lists!$B$4:$B$7</x:formula1>
@@ -6178,10 +6502,19 @@
     <x:dataValidation type="list" sqref="AS4:AS103">
       <x:formula1>Lists!$R$4:$R$5</x:formula1>
     </x:dataValidation>
+    <x:dataValidation type="list" sqref="AT4:AT103">
+      <x:formula1>Lists!$N$4:$N$57</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="AU4:AU103">
+      <x:formula1>Lists!$S$4:$S$9</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="AV4:AV103">
+      <x:formula1>Lists!$T$4:$T$7</x:formula1>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d004ba12eb24f68"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R891490476a174eae"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6235,6 +6568,9 @@
     <x:col min="43" max="43" width="28" hidden="0" customWidth="1"/>
     <x:col min="44" max="44" width="28" hidden="0" customWidth="1"/>
     <x:col min="45" max="45" width="18" hidden="0" customWidth="1"/>
+    <x:col min="46" max="46" width="18" hidden="0" customWidth="1"/>
+    <x:col min="47" max="47" width="18" hidden="0" customWidth="1"/>
+    <x:col min="48" max="48" width="18" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -6285,6 +6621,9 @@
       <x:c r="AQ1" s="86"/>
       <x:c r="AR1" s="86"/>
       <x:c r="AS1" s="86"/>
+      <x:c r="AT1" s="86"/>
+      <x:c r="AU1" s="86"/>
+      <x:c r="AV1" s="86"/>
     </x:row>
     <x:row r="3" ht="45" customHeight="1">
       <x:c r="A3" s="64" t="str">
@@ -6421,6 +6760,15 @@
       </x:c>
       <x:c r="AS3" s="64" t="str">
         <x:v>confirms_no_sensitive_data</x:v>
+      </x:c>
+      <x:c r="AT3" s="64" t="str">
+        <x:v>organisation_presence_country_iso2</x:v>
+      </x:c>
+      <x:c r="AU3" s="64" t="str">
+        <x:v>organisation_presence_type</x:v>
+      </x:c>
+      <x:c r="AV3" s="64" t="str">
+        <x:v>organisation_presence_lifecycle_status</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="58" customHeight="1">
@@ -6507,6 +6855,9 @@
       </x:c>
       <x:c r="AR4" s="65" t="str"/>
       <x:c r="AS4" s="65" t="str"/>
+      <x:c r="AT4" s="65" t="str"/>
+      <x:c r="AU4" s="65" t="str"/>
+      <x:c r="AV4" s="65" t="str"/>
     </x:row>
     <x:row r="5" ht="58" customHeight="1">
       <x:c r="A5" s="65" t="str">
@@ -6596,6 +6947,9 @@
       </x:c>
       <x:c r="AR5" s="65" t="str"/>
       <x:c r="AS5" s="65" t="str"/>
+      <x:c r="AT5" s="65" t="str"/>
+      <x:c r="AU5" s="65" t="str"/>
+      <x:c r="AV5" s="65" t="str"/>
     </x:row>
     <x:row r="6" ht="58" customHeight="1">
       <x:c r="A6" s="65" t="str">
@@ -6691,6 +7045,9 @@
       <x:c r="AS6" s="65" t="str">
         <x:v>TRUE</x:v>
       </x:c>
+      <x:c r="AT6" s="65" t="str"/>
+      <x:c r="AU6" s="65" t="str"/>
+      <x:c r="AV6" s="65" t="str"/>
     </x:row>
     <x:row r="7" ht="58" customHeight="1">
       <x:c r="A7" s="65" t="str">
@@ -6764,6 +7121,9 @@
       </x:c>
       <x:c r="AR7" s="65" t="str"/>
       <x:c r="AS7" s="65" t="str"/>
+      <x:c r="AT7" s="65" t="str"/>
+      <x:c r="AU7" s="65" t="str"/>
+      <x:c r="AV7" s="65" t="str"/>
     </x:row>
     <x:row r="8" ht="58" customHeight="1">
       <x:c r="A8" s="65" t="str">
@@ -6839,6 +7199,9 @@
       </x:c>
       <x:c r="AR8" s="65" t="str"/>
       <x:c r="AS8" s="65" t="str"/>
+      <x:c r="AT8" s="65" t="str"/>
+      <x:c r="AU8" s="65" t="str"/>
+      <x:c r="AV8" s="65" t="str"/>
     </x:row>
     <x:row r="9" ht="58" customHeight="1">
       <x:c r="A9" s="65" t="str">
@@ -6916,14 +7279,97 @@
       </x:c>
       <x:c r="AR9" s="65" t="str"/>
       <x:c r="AS9" s="65" t="str"/>
+      <x:c r="AT9" s="65" t="str"/>
+      <x:c r="AU9" s="65" t="str"/>
+      <x:c r="AV9" s="65" t="str"/>
+    </x:row>
+    <x:row r="10" ht="58" customHeight="1">
+      <x:c r="A10" s="65" t="str">
+        <x:v>example-company-stated-presence</x:v>
+      </x:c>
+      <x:c r="B10" s="65" t="str">
+        <x:v>organisation_presence</x:v>
+      </x:c>
+      <x:c r="C10" s="65" t="str">
+        <x:v>Example Energy Group</x:v>
+      </x:c>
+      <x:c r="D10" s="65" t="str">
+        <x:v>org_example_group</x:v>
+      </x:c>
+      <x:c r="E10" s="65" t="str"/>
+      <x:c r="F10" s="65" t="str"/>
+      <x:c r="G10" s="65" t="str"/>
+      <x:c r="H10" s="65" t="str"/>
+      <x:c r="I10" s="65" t="str"/>
+      <x:c r="J10" s="65" t="str"/>
+      <x:c r="K10" s="65" t="str"/>
+      <x:c r="L10" s="65" t="str"/>
+      <x:c r="M10" s="65" t="str"/>
+      <x:c r="N10" s="65" t="str"/>
+      <x:c r="O10" s="65" t="str"/>
+      <x:c r="P10" s="65" t="str"/>
+      <x:c r="Q10" s="65" t="str"/>
+      <x:c r="R10" s="65" t="str"/>
+      <x:c r="S10" s="65" t="str"/>
+      <x:c r="T10" s="65" t="str"/>
+      <x:c r="U10" s="65" t="str"/>
+      <x:c r="V10" s="65" t="str"/>
+      <x:c r="W10" s="65" t="str"/>
+      <x:c r="X10" s="65" t="str"/>
+      <x:c r="Y10" s="65" t="str"/>
+      <x:c r="Z10" s="65" t="str"/>
+      <x:c r="AA10" s="65" t="str"/>
+      <x:c r="AB10" s="65" t="str"/>
+      <x:c r="AC10" s="65" t="str"/>
+      <x:c r="AD10" s="65" t="str"/>
+      <x:c r="AE10" s="65" t="str"/>
+      <x:c r="AF10" s="65" t="str"/>
+      <x:c r="AG10" s="65" t="str"/>
+      <x:c r="AH10" s="65" t="str"/>
+      <x:c r="AI10" s="65" t="str"/>
+      <x:c r="AJ10" s="65" t="str">
+        <x:v>https://example.org/where-we-work</x:v>
+      </x:c>
+      <x:c r="AK10" s="65" t="str">
+        <x:v>Where we work</x:v>
+      </x:c>
+      <x:c r="AL10" s="65" t="str">
+        <x:v>Example Energy Group</x:v>
+      </x:c>
+      <x:c r="AM10" s="65" t="str"/>
+      <x:c r="AN10" s="65" t="str">
+        <x:v>provider_authored</x:v>
+      </x:c>
+      <x:c r="AO10" s="65" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="AP10" s="65" t="str">
+        <x:v>provider_claim_only</x:v>
+      </x:c>
+      <x:c r="AQ10" s="65" t="str">
+        <x:v>Africa operations list</x:v>
+      </x:c>
+      <x:c r="AR10" s="65" t="str">
+        <x:v>Company-stated presence; not independent confirmation.</x:v>
+      </x:c>
+      <x:c r="AS10" s="65" t="str"/>
+      <x:c r="AT10" s="65" t="str">
+        <x:v>GH</x:v>
+      </x:c>
+      <x:c r="AU10" s="65" t="str">
+        <x:v>operations</x:v>
+      </x:c>
+      <x:c r="AV10" s="65" t="str">
+        <x:v>active</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:AS1"/>
+    <x:mergeCell ref="A1:AV1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R037d762b4fba411f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb99fba752bd64822"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6974,7 +7420,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="C5" s="74" t="str">
-        <x:v>Choose organisation, product, deployment, alias, corporate relationship or software relationship.</x:v>
+        <x:v>Choose organisation, product, deployment, alias, corporate relationship, software relationship or organisation presence.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="34" customHeight="1">
@@ -7172,7 +7618,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="C23" s="74" t="str">
-        <x:v>ISO date when a role, alias or relationship began, only when sourced.</x:v>
+        <x:v>ISO date when a role, alias, relationship or country presence began, only when sourced.</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="34" customHeight="1">
@@ -7183,7 +7629,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="C24" s="74" t="str">
-        <x:v>ISO date when a role, alias or relationship ended, only when sourced.</x:v>
+        <x:v>ISO date when a role, alias, relationship or country presence ended, only when sourced.</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="34" customHeight="1">
@@ -7440,14 +7886,47 @@
       </x:c>
     </x:row>
     <x:row r="48" ht="34" customHeight="1">
-      <x:c r="A48" s="75" t="str">
+      <x:c r="A48" s="72" t="str">
         <x:v>confirms_no_sensitive_data</x:v>
       </x:c>
-      <x:c r="B48" s="80" t="str">
+      <x:c r="B48" s="79" t="str">
         <x:v>Deployment</x:v>
       </x:c>
-      <x:c r="C48" s="77" t="str">
+      <x:c r="C48" s="74" t="str">
         <x:v>TRUE confirms no precise or confidential infrastructure data is included.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="34" customHeight="1">
+      <x:c r="A49" s="72" t="str">
+        <x:v>organisation_presence_country_iso2</x:v>
+      </x:c>
+      <x:c r="B49" s="79" t="str">
+        <x:v>Organisation presence</x:v>
+      </x:c>
+      <x:c r="C49" s="74" t="str">
+        <x:v>African country ISO alpha-2 code. Headquarters and origin remain separate.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="34" customHeight="1">
+      <x:c r="A50" s="72" t="str">
+        <x:v>organisation_presence_type</x:v>
+      </x:c>
+      <x:c r="B50" s="79" t="str">
+        <x:v>Organisation presence</x:v>
+      </x:c>
+      <x:c r="C50" s="74" t="str">
+        <x:v>Choose operations, project participation, office, legal entity, product deployment or product availability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="34" customHeight="1">
+      <x:c r="A51" s="75" t="str">
+        <x:v>organisation_presence_lifecycle_status</x:v>
+      </x:c>
+      <x:c r="B51" s="80" t="str">
+        <x:v>Organisation presence</x:v>
+      </x:c>
+      <x:c r="C51" s="77" t="str">
+        <x:v>Choose active, planned, historical or unknown.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7456,7 +7935,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7fcf2c8356a94ca4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc178b2d2927d4c93"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7483,6 +7962,8 @@
     <x:col min="16" max="16" width="27" hidden="0" customWidth="1"/>
     <x:col min="17" max="17" width="27" hidden="0" customWidth="1"/>
     <x:col min="18" max="18" width="27" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="27" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="27" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -7506,6 +7987,8 @@
       <x:c r="P1" s="86"/>
       <x:c r="Q1" s="86"/>
       <x:c r="R1" s="86"/>
+      <x:c r="S1" s="86"/>
+      <x:c r="T1" s="86"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="81" t="str">
@@ -7559,8 +8042,14 @@
       <x:c r="Q3" s="82" t="str">
         <x:v>evidence_status</x:v>
       </x:c>
-      <x:c r="R3" s="83" t="str">
+      <x:c r="R3" s="82" t="str">
         <x:v>boolean</x:v>
+      </x:c>
+      <x:c r="S3" s="82" t="str">
+        <x:v>organisation_presence_type</x:v>
+      </x:c>
+      <x:c r="T3" s="83" t="str">
+        <x:v>organisation_presence_lifecycle_status</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -7615,8 +8104,14 @@
       <x:c r="Q4" s="84" t="str">
         <x:v>provider_claim_only</x:v>
       </x:c>
-      <x:c r="R4" s="23" t="str">
+      <x:c r="R4" s="84" t="str">
         <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="S4" s="84" t="str">
+        <x:v>operations</x:v>
+      </x:c>
+      <x:c r="T4" s="23" t="str">
+        <x:v>active</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -7671,8 +8166,14 @@
       <x:c r="Q5" s="84" t="str">
         <x:v>public_source</x:v>
       </x:c>
-      <x:c r="R5" s="23" t="str">
+      <x:c r="R5" s="84" t="str">
         <x:v>FALSE</x:v>
+      </x:c>
+      <x:c r="S5" s="84" t="str">
+        <x:v>project_participation</x:v>
+      </x:c>
+      <x:c r="T5" s="23" t="str">
+        <x:v>planned</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -7727,7 +8228,13 @@
       <x:c r="Q6" s="84" t="str">
         <x:v>independently_evidenced</x:v>
       </x:c>
-      <x:c r="R6" s="23"/>
+      <x:c r="R6" s="84"/>
+      <x:c r="S6" s="84" t="str">
+        <x:v>office</x:v>
+      </x:c>
+      <x:c r="T6" s="23" t="str">
+        <x:v>historical</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="22" t="str">
@@ -7781,7 +8288,13 @@
       <x:c r="Q7" s="84" t="str">
         <x:v>customer_confirmed</x:v>
       </x:c>
-      <x:c r="R7" s="23"/>
+      <x:c r="R7" s="84"/>
+      <x:c r="S7" s="84" t="str">
+        <x:v>legal_entity</x:v>
+      </x:c>
+      <x:c r="T7" s="23" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="22" t="str">
@@ -7829,7 +8342,11 @@
         <x:v>aggregator</x:v>
       </x:c>
       <x:c r="Q8" s="84"/>
-      <x:c r="R8" s="23"/>
+      <x:c r="R8" s="84"/>
+      <x:c r="S8" s="84" t="str">
+        <x:v>product_deployment</x:v>
+      </x:c>
+      <x:c r="T8" s="23"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="22" t="str">
@@ -7873,10 +8390,16 @@
         <x:v>community_submission</x:v>
       </x:c>
       <x:c r="Q9" s="84"/>
-      <x:c r="R9" s="23"/>
+      <x:c r="R9" s="84"/>
+      <x:c r="S9" s="84" t="str">
+        <x:v>product_availability</x:v>
+      </x:c>
+      <x:c r="T9" s="23"/>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="22"/>
+      <x:c r="A10" s="22" t="str">
+        <x:v>organisation_presence</x:v>
+      </x:c>
       <x:c r="B10" s="84"/>
       <x:c r="C10" s="84" t="str">
         <x:v>under_review</x:v>
@@ -7909,7 +8432,9 @@
       <x:c r="O10" s="84"/>
       <x:c r="P10" s="84"/>
       <x:c r="Q10" s="84"/>
-      <x:c r="R10" s="23"/>
+      <x:c r="R10" s="84"/>
+      <x:c r="S10" s="84"/>
+      <x:c r="T10" s="23"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="22"/>
@@ -7943,7 +8468,9 @@
       <x:c r="O11" s="84"/>
       <x:c r="P11" s="84"/>
       <x:c r="Q11" s="84"/>
-      <x:c r="R11" s="23"/>
+      <x:c r="R11" s="84"/>
+      <x:c r="S11" s="84"/>
+      <x:c r="T11" s="23"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="22"/>
@@ -7973,7 +8500,9 @@
       <x:c r="O12" s="84"/>
       <x:c r="P12" s="84"/>
       <x:c r="Q12" s="84"/>
-      <x:c r="R12" s="23"/>
+      <x:c r="R12" s="84"/>
+      <x:c r="S12" s="84"/>
+      <x:c r="T12" s="23"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="22"/>
@@ -8003,7 +8532,9 @@
       <x:c r="O13" s="84"/>
       <x:c r="P13" s="84"/>
       <x:c r="Q13" s="84"/>
-      <x:c r="R13" s="23"/>
+      <x:c r="R13" s="84"/>
+      <x:c r="S13" s="84"/>
+      <x:c r="T13" s="23"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="22"/>
@@ -8031,7 +8562,9 @@
       <x:c r="O14" s="84"/>
       <x:c r="P14" s="84"/>
       <x:c r="Q14" s="84"/>
-      <x:c r="R14" s="23"/>
+      <x:c r="R14" s="84"/>
+      <x:c r="S14" s="84"/>
+      <x:c r="T14" s="23"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="22"/>
@@ -8057,7 +8590,9 @@
       <x:c r="O15" s="84"/>
       <x:c r="P15" s="84"/>
       <x:c r="Q15" s="84"/>
-      <x:c r="R15" s="23"/>
+      <x:c r="R15" s="84"/>
+      <x:c r="S15" s="84"/>
+      <x:c r="T15" s="23"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="22"/>
@@ -8083,7 +8618,9 @@
       <x:c r="O16" s="84"/>
       <x:c r="P16" s="84"/>
       <x:c r="Q16" s="84"/>
-      <x:c r="R16" s="23"/>
+      <x:c r="R16" s="84"/>
+      <x:c r="S16" s="84"/>
+      <x:c r="T16" s="23"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="22"/>
@@ -8109,7 +8646,9 @@
       <x:c r="O17" s="84"/>
       <x:c r="P17" s="84"/>
       <x:c r="Q17" s="84"/>
-      <x:c r="R17" s="23"/>
+      <x:c r="R17" s="84"/>
+      <x:c r="S17" s="84"/>
+      <x:c r="T17" s="23"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="22"/>
@@ -8133,7 +8672,9 @@
       <x:c r="O18" s="84"/>
       <x:c r="P18" s="84"/>
       <x:c r="Q18" s="84"/>
-      <x:c r="R18" s="23"/>
+      <x:c r="R18" s="84"/>
+      <x:c r="S18" s="84"/>
+      <x:c r="T18" s="23"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="22"/>
@@ -8157,7 +8698,9 @@
       <x:c r="O19" s="84"/>
       <x:c r="P19" s="84"/>
       <x:c r="Q19" s="84"/>
-      <x:c r="R19" s="23"/>
+      <x:c r="R19" s="84"/>
+      <x:c r="S19" s="84"/>
+      <x:c r="T19" s="23"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="22"/>
@@ -8181,7 +8724,9 @@
       <x:c r="O20" s="84"/>
       <x:c r="P20" s="84"/>
       <x:c r="Q20" s="84"/>
-      <x:c r="R20" s="23"/>
+      <x:c r="R20" s="84"/>
+      <x:c r="S20" s="84"/>
+      <x:c r="T20" s="23"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="22"/>
@@ -8205,7 +8750,9 @@
       <x:c r="O21" s="84"/>
       <x:c r="P21" s="84"/>
       <x:c r="Q21" s="84"/>
-      <x:c r="R21" s="23"/>
+      <x:c r="R21" s="84"/>
+      <x:c r="S21" s="84"/>
+      <x:c r="T21" s="23"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="22"/>
@@ -8229,7 +8776,9 @@
       <x:c r="O22" s="84"/>
       <x:c r="P22" s="84"/>
       <x:c r="Q22" s="84"/>
-      <x:c r="R22" s="23"/>
+      <x:c r="R22" s="84"/>
+      <x:c r="S22" s="84"/>
+      <x:c r="T22" s="23"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="22"/>
@@ -8253,7 +8802,9 @@
       <x:c r="O23" s="84"/>
       <x:c r="P23" s="84"/>
       <x:c r="Q23" s="84"/>
-      <x:c r="R23" s="23"/>
+      <x:c r="R23" s="84"/>
+      <x:c r="S23" s="84"/>
+      <x:c r="T23" s="23"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="22"/>
@@ -8277,7 +8828,9 @@
       <x:c r="O24" s="84"/>
       <x:c r="P24" s="84"/>
       <x:c r="Q24" s="84"/>
-      <x:c r="R24" s="23"/>
+      <x:c r="R24" s="84"/>
+      <x:c r="S24" s="84"/>
+      <x:c r="T24" s="23"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="22"/>
@@ -8301,7 +8854,9 @@
       <x:c r="O25" s="84"/>
       <x:c r="P25" s="84"/>
       <x:c r="Q25" s="84"/>
-      <x:c r="R25" s="23"/>
+      <x:c r="R25" s="84"/>
+      <x:c r="S25" s="84"/>
+      <x:c r="T25" s="23"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="22"/>
@@ -8325,7 +8880,9 @@
       <x:c r="O26" s="84"/>
       <x:c r="P26" s="84"/>
       <x:c r="Q26" s="84"/>
-      <x:c r="R26" s="23"/>
+      <x:c r="R26" s="84"/>
+      <x:c r="S26" s="84"/>
+      <x:c r="T26" s="23"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="22"/>
@@ -8349,7 +8906,9 @@
       <x:c r="O27" s="84"/>
       <x:c r="P27" s="84"/>
       <x:c r="Q27" s="84"/>
-      <x:c r="R27" s="23"/>
+      <x:c r="R27" s="84"/>
+      <x:c r="S27" s="84"/>
+      <x:c r="T27" s="23"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="22"/>
@@ -8373,7 +8932,9 @@
       <x:c r="O28" s="84"/>
       <x:c r="P28" s="84"/>
       <x:c r="Q28" s="84"/>
-      <x:c r="R28" s="23"/>
+      <x:c r="R28" s="84"/>
+      <x:c r="S28" s="84"/>
+      <x:c r="T28" s="23"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="22"/>
@@ -8397,7 +8958,9 @@
       <x:c r="O29" s="84"/>
       <x:c r="P29" s="84"/>
       <x:c r="Q29" s="84"/>
-      <x:c r="R29" s="23"/>
+      <x:c r="R29" s="84"/>
+      <x:c r="S29" s="84"/>
+      <x:c r="T29" s="23"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="22"/>
@@ -8421,7 +8984,9 @@
       <x:c r="O30" s="84"/>
       <x:c r="P30" s="84"/>
       <x:c r="Q30" s="84"/>
-      <x:c r="R30" s="23"/>
+      <x:c r="R30" s="84"/>
+      <x:c r="S30" s="84"/>
+      <x:c r="T30" s="23"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="22"/>
@@ -8443,7 +9008,9 @@
       <x:c r="O31" s="84"/>
       <x:c r="P31" s="84"/>
       <x:c r="Q31" s="84"/>
-      <x:c r="R31" s="23"/>
+      <x:c r="R31" s="84"/>
+      <x:c r="S31" s="84"/>
+      <x:c r="T31" s="23"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="22"/>
@@ -8465,7 +9032,9 @@
       <x:c r="O32" s="84"/>
       <x:c r="P32" s="84"/>
       <x:c r="Q32" s="84"/>
-      <x:c r="R32" s="23"/>
+      <x:c r="R32" s="84"/>
+      <x:c r="S32" s="84"/>
+      <x:c r="T32" s="23"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="22"/>
@@ -8487,7 +9056,9 @@
       <x:c r="O33" s="84"/>
       <x:c r="P33" s="84"/>
       <x:c r="Q33" s="84"/>
-      <x:c r="R33" s="23"/>
+      <x:c r="R33" s="84"/>
+      <x:c r="S33" s="84"/>
+      <x:c r="T33" s="23"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="22"/>
@@ -8509,7 +9080,9 @@
       <x:c r="O34" s="84"/>
       <x:c r="P34" s="84"/>
       <x:c r="Q34" s="84"/>
-      <x:c r="R34" s="23"/>
+      <x:c r="R34" s="84"/>
+      <x:c r="S34" s="84"/>
+      <x:c r="T34" s="23"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="22"/>
@@ -8531,7 +9104,9 @@
       <x:c r="O35" s="84"/>
       <x:c r="P35" s="84"/>
       <x:c r="Q35" s="84"/>
-      <x:c r="R35" s="23"/>
+      <x:c r="R35" s="84"/>
+      <x:c r="S35" s="84"/>
+      <x:c r="T35" s="23"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="22"/>
@@ -8553,7 +9128,9 @@
       <x:c r="O36" s="84"/>
       <x:c r="P36" s="84"/>
       <x:c r="Q36" s="84"/>
-      <x:c r="R36" s="23"/>
+      <x:c r="R36" s="84"/>
+      <x:c r="S36" s="84"/>
+      <x:c r="T36" s="23"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="22"/>
@@ -8575,7 +9152,9 @@
       <x:c r="O37" s="84"/>
       <x:c r="P37" s="84"/>
       <x:c r="Q37" s="84"/>
-      <x:c r="R37" s="23"/>
+      <x:c r="R37" s="84"/>
+      <x:c r="S37" s="84"/>
+      <x:c r="T37" s="23"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="22"/>
@@ -8597,7 +9176,9 @@
       <x:c r="O38" s="84"/>
       <x:c r="P38" s="84"/>
       <x:c r="Q38" s="84"/>
-      <x:c r="R38" s="23"/>
+      <x:c r="R38" s="84"/>
+      <x:c r="S38" s="84"/>
+      <x:c r="T38" s="23"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="22"/>
@@ -8619,7 +9200,9 @@
       <x:c r="O39" s="84"/>
       <x:c r="P39" s="84"/>
       <x:c r="Q39" s="84"/>
-      <x:c r="R39" s="23"/>
+      <x:c r="R39" s="84"/>
+      <x:c r="S39" s="84"/>
+      <x:c r="T39" s="23"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="22"/>
@@ -8641,7 +9224,9 @@
       <x:c r="O40" s="84"/>
       <x:c r="P40" s="84"/>
       <x:c r="Q40" s="84"/>
-      <x:c r="R40" s="23"/>
+      <x:c r="R40" s="84"/>
+      <x:c r="S40" s="84"/>
+      <x:c r="T40" s="23"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="22"/>
@@ -8663,7 +9248,9 @@
       <x:c r="O41" s="84"/>
       <x:c r="P41" s="84"/>
       <x:c r="Q41" s="84"/>
-      <x:c r="R41" s="23"/>
+      <x:c r="R41" s="84"/>
+      <x:c r="S41" s="84"/>
+      <x:c r="T41" s="23"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="22"/>
@@ -8685,7 +9272,9 @@
       <x:c r="O42" s="84"/>
       <x:c r="P42" s="84"/>
       <x:c r="Q42" s="84"/>
-      <x:c r="R42" s="23"/>
+      <x:c r="R42" s="84"/>
+      <x:c r="S42" s="84"/>
+      <x:c r="T42" s="23"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="22"/>
@@ -8707,7 +9296,9 @@
       <x:c r="O43" s="84"/>
       <x:c r="P43" s="84"/>
       <x:c r="Q43" s="84"/>
-      <x:c r="R43" s="23"/>
+      <x:c r="R43" s="84"/>
+      <x:c r="S43" s="84"/>
+      <x:c r="T43" s="23"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="22"/>
@@ -8729,7 +9320,9 @@
       <x:c r="O44" s="84"/>
       <x:c r="P44" s="84"/>
       <x:c r="Q44" s="84"/>
-      <x:c r="R44" s="23"/>
+      <x:c r="R44" s="84"/>
+      <x:c r="S44" s="84"/>
+      <x:c r="T44" s="23"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="22"/>
@@ -8751,7 +9344,9 @@
       <x:c r="O45" s="84"/>
       <x:c r="P45" s="84"/>
       <x:c r="Q45" s="84"/>
-      <x:c r="R45" s="23"/>
+      <x:c r="R45" s="84"/>
+      <x:c r="S45" s="84"/>
+      <x:c r="T45" s="23"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="22"/>
@@ -8773,7 +9368,9 @@
       <x:c r="O46" s="84"/>
       <x:c r="P46" s="84"/>
       <x:c r="Q46" s="84"/>
-      <x:c r="R46" s="23"/>
+      <x:c r="R46" s="84"/>
+      <x:c r="S46" s="84"/>
+      <x:c r="T46" s="23"/>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="22"/>
@@ -8795,7 +9392,9 @@
       <x:c r="O47" s="84"/>
       <x:c r="P47" s="84"/>
       <x:c r="Q47" s="84"/>
-      <x:c r="R47" s="23"/>
+      <x:c r="R47" s="84"/>
+      <x:c r="S47" s="84"/>
+      <x:c r="T47" s="23"/>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="22"/>
@@ -8817,7 +9416,9 @@
       <x:c r="O48" s="84"/>
       <x:c r="P48" s="84"/>
       <x:c r="Q48" s="84"/>
-      <x:c r="R48" s="23"/>
+      <x:c r="R48" s="84"/>
+      <x:c r="S48" s="84"/>
+      <x:c r="T48" s="23"/>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="22"/>
@@ -8839,7 +9440,9 @@
       <x:c r="O49" s="84"/>
       <x:c r="P49" s="84"/>
       <x:c r="Q49" s="84"/>
-      <x:c r="R49" s="23"/>
+      <x:c r="R49" s="84"/>
+      <x:c r="S49" s="84"/>
+      <x:c r="T49" s="23"/>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="22"/>
@@ -8861,7 +9464,9 @@
       <x:c r="O50" s="84"/>
       <x:c r="P50" s="84"/>
       <x:c r="Q50" s="84"/>
-      <x:c r="R50" s="23"/>
+      <x:c r="R50" s="84"/>
+      <x:c r="S50" s="84"/>
+      <x:c r="T50" s="23"/>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="22"/>
@@ -8883,7 +9488,9 @@
       <x:c r="O51" s="84"/>
       <x:c r="P51" s="84"/>
       <x:c r="Q51" s="84"/>
-      <x:c r="R51" s="23"/>
+      <x:c r="R51" s="84"/>
+      <x:c r="S51" s="84"/>
+      <x:c r="T51" s="23"/>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="22"/>
@@ -8905,7 +9512,9 @@
       <x:c r="O52" s="84"/>
       <x:c r="P52" s="84"/>
       <x:c r="Q52" s="84"/>
-      <x:c r="R52" s="23"/>
+      <x:c r="R52" s="84"/>
+      <x:c r="S52" s="84"/>
+      <x:c r="T52" s="23"/>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="22"/>
@@ -8927,7 +9536,9 @@
       <x:c r="O53" s="84"/>
       <x:c r="P53" s="84"/>
       <x:c r="Q53" s="84"/>
-      <x:c r="R53" s="23"/>
+      <x:c r="R53" s="84"/>
+      <x:c r="S53" s="84"/>
+      <x:c r="T53" s="23"/>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="22"/>
@@ -8949,7 +9560,9 @@
       <x:c r="O54" s="84"/>
       <x:c r="P54" s="84"/>
       <x:c r="Q54" s="84"/>
-      <x:c r="R54" s="23"/>
+      <x:c r="R54" s="84"/>
+      <x:c r="S54" s="84"/>
+      <x:c r="T54" s="23"/>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="22"/>
@@ -8971,7 +9584,9 @@
       <x:c r="O55" s="84"/>
       <x:c r="P55" s="84"/>
       <x:c r="Q55" s="84"/>
-      <x:c r="R55" s="23"/>
+      <x:c r="R55" s="84"/>
+      <x:c r="S55" s="84"/>
+      <x:c r="T55" s="23"/>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="22"/>
@@ -8993,7 +9608,9 @@
       <x:c r="O56" s="84"/>
       <x:c r="P56" s="84"/>
       <x:c r="Q56" s="84"/>
-      <x:c r="R56" s="23"/>
+      <x:c r="R56" s="84"/>
+      <x:c r="S56" s="84"/>
+      <x:c r="T56" s="23"/>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="24"/>
@@ -9015,11 +9632,13 @@
       <x:c r="O57" s="85"/>
       <x:c r="P57" s="85"/>
       <x:c r="Q57" s="85"/>
-      <x:c r="R57" s="25"/>
+      <x:c r="R57" s="85"/>
+      <x:c r="S57" s="85"/>
+      <x:c r="T57" s="25"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:R1"/>
+    <x:mergeCell ref="A1:T1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>